<commit_message>
Corrige resumen de la matriz de pruebas
</commit_message>
<xml_diff>
--- a/Pruebas/Matriz_de_pruebas_WorkTrack.xlsx
+++ b/Pruebas/Matriz_de_pruebas_WorkTrack.xlsx
@@ -459,8 +459,8 @@
         <x:v>Con observación</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:f>COUNTIF(G13:G58,"*observación*")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF(G13:G58,"Aprobado con observación")</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10"/>

</xml_diff>